<commit_message>
add mea. 030040-0008A, F004, F008
</commit_message>
<xml_diff>
--- a/Measurements/FAR_template_v2.xlsx
+++ b/Measurements/FAR_template_v2.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\manoe\Meng\solidworks\Measurements\05426 PIN, front shock\batch02\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\manoe\Meng\solidworks\Measurements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C182DC9-0253-4FD7-9C20-30F275106B4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFAC8A27-E9C4-44FD-998C-9D61110187EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{32BFC42B-CD3D-49FE-8254-52B3F518DB85}"/>
   </bookViews>
@@ -569,14 +569,14 @@
     <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="2" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="166" fontId="7" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -599,7 +599,7 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFFFCC"/>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1871,7 +1871,7 @@
       <c r="F1" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="G1" s="34" t="s">
+      <c r="G1" s="36" t="s">
         <v>22</v>
       </c>
       <c r="H1" s="17"/>
@@ -1900,7 +1900,7 @@
       <c r="F2" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="G2" s="34"/>
+      <c r="G2" s="36"/>
       <c r="H2" s="17"/>
       <c r="I2" s="15"/>
       <c r="J2" s="15"/>
@@ -1926,7 +1926,7 @@
         <v>5</v>
       </c>
       <c r="F3" s="12"/>
-      <c r="G3" s="34"/>
+      <c r="G3" s="36"/>
       <c r="H3" s="18"/>
       <c r="I3" s="16"/>
       <c r="J3" s="16"/>
@@ -2157,11 +2157,11 @@
       <c r="B9" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="35">
+      <c r="C9" s="34">
         <v>0.17699999999999999</v>
       </c>
-      <c r="D9" s="36"/>
-      <c r="E9" s="36"/>
+      <c r="D9" s="35"/>
+      <c r="E9" s="35"/>
       <c r="F9" s="3">
         <f t="shared" si="0"/>
         <v>0.17699999999999999</v>
@@ -2451,7 +2451,7 @@
   <mergeCells count="1">
     <mergeCell ref="G1:G3"/>
   </mergeCells>
-  <conditionalFormatting sqref="I5:M8 I10:M15">
+  <conditionalFormatting sqref="I5:M15">
     <cfRule type="cellIs" dxfId="1" priority="22" operator="notBetween">
       <formula>$G5</formula>
       <formula>$F5</formula>

</xml_diff>

<commit_message>
add measusrements, add drawing for tube
</commit_message>
<xml_diff>
--- a/Measurements/FAR_template_v2.xlsx
+++ b/Measurements/FAR_template_v2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\manoe\Meng\solidworks\Measurements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFAC8A27-E9C4-44FD-998C-9D61110187EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A076EF17-7248-4F92-B602-64CB396B3C97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{32BFC42B-CD3D-49FE-8254-52B3F518DB85}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{32BFC42B-CD3D-49FE-8254-52B3F518DB85}"/>
   </bookViews>
   <sheets>
     <sheet name="FAI" sheetId="3" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="Tolerance Table " sheetId="5" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">FAI!$A$5:$M$36</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">FAI!$A$5:$M$35</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Print Page 1'!$A$1:$Q$40</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="30">
   <si>
     <t>Customer</t>
   </si>
@@ -84,9 +84,6 @@
   </si>
   <si>
     <t>Length</t>
-  </si>
-  <si>
-    <t>VMM</t>
   </si>
   <si>
     <t>Type        (Diameter Length Position etc.)</t>
@@ -132,37 +129,13 @@
     <t>Angle (Chamfer)</t>
   </si>
   <si>
-    <t>7a</t>
-  </si>
-  <si>
     <t>Length (Chamfer)</t>
   </si>
   <si>
-    <t>7b</t>
-  </si>
-  <si>
-    <t>Radius (Fillet)</t>
-  </si>
-  <si>
     <t>Inch</t>
   </si>
   <si>
-    <t>8a</t>
-  </si>
-  <si>
-    <t>8b</t>
-  </si>
-  <si>
-    <t>05426</t>
-  </si>
-  <si>
-    <t>Pin, Front Shock</t>
-  </si>
-  <si>
     <t xml:space="preserve"> </t>
-  </si>
-  <si>
-    <t>2/25/2026</t>
   </si>
 </sst>
 </file>
@@ -274,7 +247,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -466,11 +439,24 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="166" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -545,9 +531,6 @@
     <xf numFmtId="164" fontId="9" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -563,9 +546,6 @@
     <xf numFmtId="1" fontId="4" fillId="3" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="4" fillId="3" borderId="14" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -575,24 +555,26 @@
     <xf numFmtId="165" fontId="1" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="6" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="3" borderId="14" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="4" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <font>
         <color rgb="FFFF0000"/>
@@ -635,7 +617,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
-      <xdr:colOff>3623</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>2602</xdr:rowOff>
     </xdr:to>
@@ -660,8 +642,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6381750" y="0"/>
-          <a:ext cx="3690937" cy="1094354"/>
+          <a:off x="6377609" y="0"/>
+          <a:ext cx="3321326" cy="1104189"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -680,50 +662,6 @@
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>96710</xdr:colOff>
-      <xdr:row>42</xdr:row>
-      <xdr:rowOff>1117</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{96EB7E65-EA31-BD4B-711E-849EBBF25A88}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="571500"/>
-          <a:ext cx="10459910" cy="8002117"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>4</xdr:col>
@@ -1461,60 +1399,6 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>28575</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>153976</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E4C11B6C-CFF2-7AAE-5A10-F9C37E73F638}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="4905375" cy="1106476"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:solidFill>
-            <a:schemeClr val="tx1"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1838,7 +1722,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" style="1" customWidth="1"/>
@@ -1849,10 +1733,7 @@
     <col min="6" max="6" width="8.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.5703125" style="1" customWidth="1"/>
     <col min="8" max="8" width="11.28515625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="8.85546875" style="1" customWidth="1"/>
-    <col min="10" max="11" width="8.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.85546875" style="1" customWidth="1"/>
-    <col min="13" max="13" width="8.7109375" style="1" customWidth="1"/>
+    <col min="9" max="13" width="7.7109375" style="1" customWidth="1"/>
     <col min="14" max="16384" width="8.7109375" style="1"/>
   </cols>
   <sheetData>
@@ -1862,17 +1743,18 @@
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D1" s="24"/>
       <c r="E1" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="26" t="s">
-        <v>38</v>
+      <c r="F1" s="34">
+        <f ca="1">TODAY()</f>
+        <v>46097</v>
       </c>
       <c r="G1" s="36" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H1" s="17"/>
       <c r="I1" s="15"/>
@@ -1885,11 +1767,9 @@
       <c r="A2" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="8" t="s">
-        <v>36</v>
-      </c>
+      <c r="B2" s="8"/>
       <c r="C2" s="9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D2" s="13">
         <v>5</v>
@@ -1898,9 +1778,9 @@
         <v>3</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="G2" s="36"/>
+        <v>25</v>
+      </c>
+      <c r="G2" s="37"/>
       <c r="H2" s="17"/>
       <c r="I2" s="15"/>
       <c r="J2" s="15"/>
@@ -1910,23 +1790,21 @@
       <c r="N2"/>
     </row>
     <row r="3" spans="1:14" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="27" t="s">
+      <c r="A3" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="33" t="s">
-        <v>35</v>
-      </c>
+      <c r="B3" s="31"/>
       <c r="C3" s="20" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="E3" s="10" t="s">
         <v>5</v>
       </c>
       <c r="F3" s="12"/>
-      <c r="G3" s="36"/>
+      <c r="G3" s="38"/>
       <c r="H3" s="18"/>
       <c r="I3" s="16"/>
       <c r="J3" s="16"/>
@@ -1934,48 +1812,48 @@
       <c r="L3" s="22"/>
       <c r="M3" s="16"/>
     </row>
-    <row r="4" spans="1:14" ht="60" x14ac:dyDescent="0.25">
-      <c r="A4" s="28" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" s="29" t="s">
+    <row r="4" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A4" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="28" t="s">
+      <c r="B4" s="28" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="30" t="s">
+      <c r="D4" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="30" t="s">
+      <c r="E4" s="29" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="28" t="s">
+      <c r="F4" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="G4" s="31" t="s">
+      <c r="G4" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="H4" s="31" t="s">
+      <c r="H4" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="I4" s="32" t="s">
+      <c r="I4" s="35" t="s">
+        <v>18</v>
+      </c>
+      <c r="J4" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="J4" s="32" t="s">
+      <c r="K4" s="35" t="s">
         <v>20</v>
       </c>
-      <c r="K4" s="32" t="s">
-        <v>21</v>
-      </c>
-      <c r="L4" s="32" t="s">
+      <c r="L4" s="35" t="s">
+        <v>23</v>
+      </c>
+      <c r="M4" s="35" t="s">
         <v>24</v>
       </c>
-      <c r="M4" s="32" t="s">
-        <v>25</v>
-      </c>
       <c r="N4" s="1" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
@@ -1985,41 +1863,23 @@
       <c r="B5" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="6">
-        <v>6.1849999999999996</v>
-      </c>
-      <c r="D5" s="3">
-        <v>2.5000000000000001E-2</v>
-      </c>
-      <c r="E5" s="3">
-        <v>2.5000000000000001E-2</v>
-      </c>
+      <c r="C5" s="6"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
       <c r="F5" s="3">
         <f>C5+D5</f>
-        <v>6.21</v>
+        <v>0</v>
       </c>
       <c r="G5" s="3">
         <f>C5-E5</f>
-        <v>6.1599999999999993</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I5" s="2">
-        <v>6.1890000000000001</v>
-      </c>
-      <c r="J5" s="2">
-        <v>6.1870000000000003</v>
-      </c>
-      <c r="K5" s="2">
-        <v>6.1740000000000004</v>
-      </c>
-      <c r="L5" s="2">
-        <v>6.1580000000000004</v>
-      </c>
-      <c r="M5" s="2">
-        <v>6.1779999999999999</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="H5" s="3"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
+      <c r="K5" s="2"/>
+      <c r="L5" s="2"/>
+      <c r="M5" s="2"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
@@ -2028,41 +1888,23 @@
       <c r="B6" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="6">
-        <v>0.81</v>
-      </c>
-      <c r="D6" s="3">
-        <v>0.01</v>
-      </c>
-      <c r="E6" s="3">
-        <v>0.01</v>
-      </c>
+      <c r="C6" s="6"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
       <c r="F6" s="3">
         <f>C6+D6</f>
-        <v>0.82000000000000006</v>
+        <v>0</v>
       </c>
       <c r="G6" s="3">
         <f>C6-E6</f>
-        <v>0.8</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I6" s="2">
-        <v>0.80900000000000005</v>
-      </c>
-      <c r="J6" s="2">
-        <v>0.80920000000000003</v>
-      </c>
-      <c r="K6" s="2">
-        <v>0.81120000000000003</v>
-      </c>
-      <c r="L6" s="2">
-        <v>0.81100000000000005</v>
-      </c>
-      <c r="M6" s="2">
-        <v>0.81069999999999998</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="H6" s="3"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2"/>
+      <c r="L6" s="2"/>
+      <c r="M6" s="2"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="4">
@@ -2071,41 +1913,23 @@
       <c r="B7" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="6">
-        <v>0.19950000000000001</v>
-      </c>
-      <c r="D7" s="3">
-        <v>9.4999999999999998E-3</v>
-      </c>
-      <c r="E7" s="3">
-        <v>9.4999999999999998E-3</v>
-      </c>
+      <c r="C7" s="6"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
       <c r="F7" s="3">
         <f t="shared" ref="F7:F11" si="0">C7+D7</f>
-        <v>0.20900000000000002</v>
+        <v>0</v>
       </c>
       <c r="G7" s="3">
         <f t="shared" ref="G7:G11" si="1">C7-E7</f>
-        <v>0.19</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I7" s="2">
-        <v>0.20710000000000001</v>
-      </c>
-      <c r="J7" s="2">
-        <v>0.2014</v>
-      </c>
-      <c r="K7" s="2">
-        <v>0.20899999999999999</v>
-      </c>
-      <c r="L7" s="2">
-        <v>0.1996</v>
-      </c>
-      <c r="M7" s="2">
-        <v>0.1933</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="H7" s="3"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="4">
@@ -2114,41 +1938,23 @@
       <c r="B8" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="6">
-        <v>3.3849999999999998</v>
-      </c>
-      <c r="D8" s="3">
-        <v>0.01</v>
-      </c>
-      <c r="E8" s="3">
-        <v>0.01</v>
-      </c>
+      <c r="C8" s="6"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
       <c r="F8" s="3">
         <f t="shared" si="0"/>
-        <v>3.3949999999999996</v>
+        <v>0</v>
       </c>
       <c r="G8" s="3">
         <f t="shared" si="1"/>
-        <v>3.375</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I8" s="2">
-        <v>3.387</v>
-      </c>
-      <c r="J8" s="2">
-        <v>3.3864000000000001</v>
-      </c>
-      <c r="K8" s="2">
-        <v>3.3868999999999998</v>
-      </c>
-      <c r="L8" s="2">
-        <v>3.3889999999999998</v>
-      </c>
-      <c r="M8" s="2">
-        <v>3.3908999999999998</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="H8" s="3"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
+      <c r="K8" s="2"/>
+      <c r="L8" s="2"/>
+      <c r="M8" s="2"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="4">
@@ -2157,37 +1963,23 @@
       <c r="B9" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="34">
-        <v>0.17699999999999999</v>
-      </c>
-      <c r="D9" s="35"/>
-      <c r="E9" s="35"/>
+      <c r="C9" s="32"/>
+      <c r="D9" s="33"/>
+      <c r="E9" s="33"/>
       <c r="F9" s="3">
         <f t="shared" si="0"/>
-        <v>0.17699999999999999</v>
+        <v>0</v>
       </c>
       <c r="G9" s="3">
         <f t="shared" si="1"/>
-        <v>0.17699999999999999</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I9" s="2">
-        <v>0.1638</v>
-      </c>
-      <c r="J9" s="2">
-        <v>0.16270000000000001</v>
-      </c>
-      <c r="K9" s="2">
-        <v>0.15920000000000001</v>
-      </c>
-      <c r="L9" s="2">
-        <v>0.157</v>
-      </c>
-      <c r="M9" s="2">
-        <v>0.1615</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="H9" s="3"/>
+      <c r="I9" s="2"/>
+      <c r="J9" s="2"/>
+      <c r="K9" s="2"/>
+      <c r="L9" s="2"/>
+      <c r="M9" s="2"/>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="4">
@@ -2196,263 +1988,130 @@
       <c r="B10" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="6">
-        <v>3.2250000000000001</v>
-      </c>
-      <c r="D10" s="3">
-        <v>0.01</v>
-      </c>
-      <c r="E10" s="3">
-        <v>0.01</v>
-      </c>
+      <c r="C10" s="6"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
       <c r="F10" s="3">
         <f t="shared" si="0"/>
-        <v>3.2349999999999999</v>
+        <v>0</v>
       </c>
       <c r="G10" s="3">
         <f t="shared" si="1"/>
-        <v>3.2150000000000003</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I10" s="2">
-        <v>3.2235</v>
-      </c>
-      <c r="J10" s="2">
-        <v>3.2176</v>
-      </c>
-      <c r="K10" s="2">
-        <v>3.2153</v>
-      </c>
-      <c r="L10" s="2">
-        <v>3.2185999999999999</v>
-      </c>
-      <c r="M10" s="2">
-        <v>3.2282000000000002</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="H10" s="3"/>
+      <c r="I10" s="2"/>
+      <c r="J10" s="2"/>
+      <c r="K10" s="2"/>
+      <c r="L10" s="2"/>
+      <c r="M10" s="2"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
-        <v>28</v>
+      <c r="A11" s="4">
+        <v>7</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="C11" s="6">
-        <v>0.06</v>
-      </c>
-      <c r="D11" s="3">
-        <v>0.01</v>
-      </c>
-      <c r="E11" s="3">
-        <v>0.01</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="C11" s="6"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
       <c r="F11" s="3">
         <f t="shared" si="0"/>
-        <v>6.9999999999999993E-2</v>
+        <v>0</v>
       </c>
       <c r="G11" s="3">
         <f t="shared" si="1"/>
-        <v>4.9999999999999996E-2</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I11" s="2">
-        <v>6.9599999999999995E-2</v>
-      </c>
-      <c r="J11" s="2">
-        <v>5.5599999999999997E-2</v>
-      </c>
-      <c r="K11" s="2">
-        <v>6.6199999999999995E-2</v>
-      </c>
-      <c r="L11" s="2">
-        <v>5.8099999999999999E-2</v>
-      </c>
-      <c r="M11" s="2">
-        <v>5.1499999999999997E-2</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="H11" s="3"/>
+      <c r="I11" s="2"/>
+      <c r="J11" s="2"/>
+      <c r="K11" s="2"/>
+      <c r="L11" s="2"/>
+      <c r="M11" s="2"/>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
-        <v>30</v>
+      <c r="A12" s="4">
+        <v>8</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="C12" s="6">
-        <v>45</v>
-      </c>
-      <c r="D12" s="3">
-        <v>1</v>
-      </c>
-      <c r="E12" s="3">
-        <v>1</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="C12" s="6"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
       <c r="F12" s="3">
-        <f t="shared" ref="F12:F15" si="2">C12+D12</f>
-        <v>46</v>
+        <f t="shared" ref="F12:F14" si="2">C12+D12</f>
+        <v>0</v>
       </c>
       <c r="G12" s="3">
-        <f t="shared" ref="G12:G15" si="3">C12-E12</f>
-        <v>44</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I12" s="2">
-        <v>44.652500000000003</v>
-      </c>
-      <c r="J12" s="2">
-        <v>44.400199999999998</v>
-      </c>
-      <c r="K12" s="2">
-        <v>44.2117</v>
-      </c>
-      <c r="L12" s="2">
-        <v>44.096499999999999</v>
-      </c>
-      <c r="M12" s="2">
-        <v>44.815300000000001</v>
-      </c>
+        <f t="shared" ref="G12:G14" si="3">C12-E12</f>
+        <v>0</v>
+      </c>
+      <c r="H12" s="3"/>
+      <c r="I12" s="2"/>
+      <c r="J12" s="2"/>
+      <c r="K12" s="2"/>
+      <c r="L12" s="2"/>
+      <c r="M12" s="2"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
-        <v>33</v>
+      <c r="A13" s="4">
+        <v>9</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="C13" s="6">
-        <v>7.5999999999999998E-2</v>
-      </c>
-      <c r="D13" s="3">
-        <v>0.01</v>
-      </c>
-      <c r="E13" s="3">
-        <v>0.01</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="C13" s="6"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
       <c r="F13" s="3">
         <f t="shared" si="2"/>
-        <v>8.5999999999999993E-2</v>
+        <v>0</v>
       </c>
       <c r="G13" s="3">
         <f t="shared" si="3"/>
-        <v>6.6000000000000003E-2</v>
-      </c>
-      <c r="H13" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I13" s="2">
-        <v>9.98E-2</v>
-      </c>
-      <c r="J13" s="2">
-        <v>8.9700000000000002E-2</v>
-      </c>
-      <c r="K13" s="2">
-        <v>9.64E-2</v>
-      </c>
-      <c r="L13" s="2">
-        <v>6.7299999999999999E-2</v>
-      </c>
-      <c r="M13" s="2">
-        <v>8.5300000000000001E-2</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="H13" s="3"/>
+      <c r="I13" s="2"/>
+      <c r="J13" s="2"/>
+      <c r="K13" s="2"/>
+      <c r="L13" s="2"/>
+      <c r="M13" s="2"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
-        <v>34</v>
+      <c r="A14" s="4">
+        <v>10</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="C14" s="6">
-        <v>15</v>
-      </c>
-      <c r="D14" s="3">
-        <v>1</v>
-      </c>
-      <c r="E14" s="3">
-        <v>1</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="C14" s="6"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
       <c r="F14" s="3">
         <f t="shared" si="2"/>
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="G14" s="3">
         <f t="shared" si="3"/>
-        <v>14</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I14" s="2">
-        <v>15.154299999999999</v>
-      </c>
-      <c r="J14" s="2">
-        <v>15.324999999999999</v>
-      </c>
-      <c r="K14" s="2">
-        <v>15.224</v>
-      </c>
-      <c r="L14" s="2">
-        <v>15.22</v>
-      </c>
-      <c r="M14" s="2">
-        <v>15.145200000000001</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" s="4">
-        <v>9</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="C15" s="6">
-        <v>1.7500000000000002E-2</v>
-      </c>
-      <c r="D15" s="3">
-        <v>7.4999999999999997E-3</v>
-      </c>
-      <c r="E15" s="3">
-        <v>7.4999999999999997E-3</v>
-      </c>
-      <c r="F15" s="3">
-        <f t="shared" si="2"/>
-        <v>2.5000000000000001E-2</v>
-      </c>
-      <c r="G15" s="3">
-        <f t="shared" si="3"/>
-        <v>1.0000000000000002E-2</v>
-      </c>
-      <c r="H15" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I15" s="2">
-        <v>3.1099999999999999E-2</v>
-      </c>
-      <c r="J15" s="2">
-        <v>2.7799999999999998E-2</v>
-      </c>
-      <c r="K15" s="2">
-        <v>2.76E-2</v>
-      </c>
-      <c r="L15" s="2">
-        <v>1.9900000000000001E-2</v>
-      </c>
-      <c r="M15" s="2">
-        <v>1.1900000000000001E-2</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="H14" s="3"/>
+      <c r="I14" s="2"/>
+      <c r="J14" s="2"/>
+      <c r="K14" s="2"/>
+      <c r="L14" s="2"/>
+      <c r="M14" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="G1:G3"/>
   </mergeCells>
-  <conditionalFormatting sqref="I5:M15">
-    <cfRule type="cellIs" dxfId="1" priority="22" operator="notBetween">
+  <conditionalFormatting sqref="I5:M14">
+    <cfRule type="cellIs" dxfId="0" priority="22" operator="notBetween">
       <formula>$G5</formula>
       <formula>$F5</formula>
     </cfRule>
@@ -2480,6 +2139,5 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add new measurement and model
</commit_message>
<xml_diff>
--- a/Measurements/FAR_template_v2.xlsx
+++ b/Measurements/FAR_template_v2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\manoe\Meng\solidworks\Measurements\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\manoe\Meng\ManoEng\Measurements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A076EF17-7248-4F92-B602-64CB396B3C97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31D4A6E7-3156-4CBC-9812-4DFD63BEB109}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{32BFC42B-CD3D-49FE-8254-52B3F518DB85}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{32BFC42B-CD3D-49FE-8254-52B3F518DB85}"/>
   </bookViews>
   <sheets>
     <sheet name="FAI" sheetId="3" r:id="rId1"/>
@@ -574,7 +574,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
     <dxf>
       <font>
         <color rgb="FFFF0000"/>
@@ -582,6 +582,16 @@
       <fill>
         <patternFill>
           <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1751,7 +1761,7 @@
       </c>
       <c r="F1" s="34">
         <f ca="1">TODAY()</f>
-        <v>46097</v>
+        <v>46119</v>
       </c>
       <c r="G1" s="36" t="s">
         <v>21</v>
@@ -2111,7 +2121,7 @@
     <mergeCell ref="G1:G3"/>
   </mergeCells>
   <conditionalFormatting sqref="I5:M14">
-    <cfRule type="cellIs" dxfId="0" priority="22" operator="notBetween">
+    <cfRule type="cellIs" dxfId="1" priority="22" operator="notBetween">
       <formula>$G5</formula>
       <formula>$F5</formula>
     </cfRule>

</xml_diff>